<commit_message>
share the WGCNA engine between trees, it never referenced group anyway
</commit_message>
<xml_diff>
--- a/03_Analysis/categorical/03_WGCNA/c_data/WGCNA_source_data.xlsx
+++ b/03_Analysis/categorical/03_WGCNA/c_data/WGCNA_source_data.xlsx
@@ -6293,7 +6293,7 @@
     <t xml:space="preserve">module movement</t>
   </si>
   <si>
-    <t xml:space="preserve">limma::fry, modules as the index, on the 03_DEP design with subject block and duplicateCorrelation</t>
+    <t xml:space="preserve">limma::fry, modules as the index, on the stage 03 design with subject block and duplicateCorrelation</t>
   </si>
   <si>
     <t xml:space="preserve">not fgsea</t>
@@ -6311,7 +6311,7 @@
     <t xml:space="preserve">source</t>
   </si>
   <si>
-    <t xml:space="preserve">02_Normalization/imputation (missForest), 00_input/c_data/phenotype.csv, 03_DEP/a_non_imputed</t>
+    <t xml:space="preserve">02_Normalization/imputation (missForest), 00_input/c_data/phenotype.csv, 03_Features/01_Proteins</t>
   </si>
 </sst>
 </file>

</xml_diff>